<commit_message>
GovGrant-Approval Decision update as per FW pkg
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B69143-4346-448D-B862-63548E1446BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F32CBC7-3D94-4F94-A8A8-E5052F7DC704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
@@ -1284,10 +1284,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -1295,7 +1295,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -1306,7 +1306,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -1317,18 +1317,18 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B9" s="5"/>
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B8" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{7EE9E90B-967F-44F2-8381-163CD7361D89}"/>
+    <hyperlink ref="C7" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{7EE9E90B-967F-44F2-8381-163CD7361D89}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>